<commit_message>
PivotTable Fields pane: tick fields, drag them between filters, columns, rows and values, filter their items and change how values are summarised, each an undoable step saved as the pivot's new definition and cache
</commit_message>
<xml_diff>
--- a/examples/demo/public/samples/pivot.xlsx
+++ b/examples/demo/public/samples/pivot.xlsx
@@ -59,13 +59,13 @@
     <t>Units by region (pivot table)</t>
   </si>
   <si>
+    <t>Edit the Data sheet and the pivot table follows; right-click it and choose Show Field List to change its fields.</t>
+  </si>
+  <si>
     <t>Row Labels</t>
   </si>
   <si>
     <t>Sum of Units</t>
-  </si>
-  <si>
-    <t>Edit units on the Data sheet; the pivot refreshes when the file is opened in Excel.</t>
   </si>
   <si>
     <t>Grand Total</t>
@@ -2385,19 +2385,21 @@
     <col min="2" max="2" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D1" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B3" t="s">
-        <v>15</v>
-      </c>
-      <c r="D3" t="s">
         <v>16</v>
       </c>
     </row>

</xml_diff>